<commit_message>
prompt engineering to get 88% and 94% precision and recall
</commit_message>
<xml_diff>
--- a/output/test30_consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
+++ b/output/test30_consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
@@ -478,49 +478,56 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HGNC:2895</t>
+          <t>HGNC:10963</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ENSG00000135960</t>
+          <t>ENSG00000175003</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GENE ID:10913</t>
+          <t>GENE ID:6580</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EDAR</t>
+          <t>SLC22A1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>EDA1R</t>
+          <t>HOCT1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ectodysplasin A receptor</t>
+          <t>solute carrier family 22 member 1</t>
         </is>
       </c>
       <c r="G2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: EDA1R
-    HGNC record ID: HGNC:2895
-    Primary gene symbol: EDAR
-    Official HGNC gene name: ectodysplasin A receptor
+    Alias gene symbol: HOCT1
+    HGNC record ID: HGNC:10963
+    Primary gene symbol: SLC22A1
+    Official HGNC gene name: solute carrier family 22 member 1
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -531,16 +538,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "EDA1R",
-    "primary_gene_symbol": "EDAR",
-    "name": "ectodysplasin A receptor",
+    "hgnc_id:"HGNC:10963"
+    "alias_symbol": "HOCT1",
+    "primary_gene_symbol": "SLC22A1",
+    "name": "solute carrier family 22 member 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -548,11 +555,11 @@
       <c r="I2" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "EDA1R",
-"primary_gene_symbol": "EDAR",
-"name": "ectodysplasin A receptor",
-"alternate_abbreviation": "TRUE"
+"hgnc_id": "HGNC:10963",
+"alias_symbol": "HOCT1",
+"primary_gene_symbol": "SLC22A1",
+"name": "solute carrier family 22 member 1",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -560,32 +567,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HGNC:13243</t>
+          <t>HGNC:8609</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ENSG00000105983</t>
+          <t>ENSG00000140694</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GENE ID:64327</t>
+          <t>GENE ID:5073</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LMBR1</t>
+          <t>PARN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PPD2</t>
+          <t>DKCB6</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>limb development membrane protein 1</t>
+          <t>poly(A)-specific ribonuclease</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -595,14 +602,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: PPD2
-    HGNC record ID: HGNC:13243
-    Primary gene symbol: LMBR1
-    Official HGNC gene name: limb development membrane protein 1
+    Alias gene symbol: DKCB6
+    HGNC record ID: HGNC:8609
+    Primary gene symbol: PARN
+    Official HGNC gene name: poly(A)-specific ribonuclease
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -613,16 +627,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "PPD2",
-    "primary_gene_symbol": "LMBR1",
-    "name": "limb development membrane protein 1",
+    "hgnc_id:"HGNC:8609"
+    "alias_symbol": "DKCB6",
+    "primary_gene_symbol": "PARN",
+    "name": "poly(A)-specific ribonuclease",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -630,10 +644,10 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "PPD2",
-"primary_gene_symbol": "LMBR1",
-"name": "limb development membrane protein 1",
+"hgnc_id": "HGNC:8609",
+"alias_symbol": "DKCB6",
+"primary_gene_symbol": "PARN",
+"name": "poly(A)-specific ribonuclease",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -642,32 +656,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HGNC:11630</t>
+          <t>HGNC:4055</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENSG00000275410</t>
+          <t>ENSG00000196419</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GENE ID:6928</t>
+          <t>GENE ID:2547</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>HNF1B</t>
+          <t>XRCC6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HPC11</t>
+          <t>D22S671</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>HNF1 homeobox B</t>
+          <t>X-ray repair cross complementing 6</t>
         </is>
       </c>
       <c r="G4" t="b">
@@ -677,14 +691,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: HPC11
-    HGNC record ID: HGNC:11630
-    Primary gene symbol: HNF1B
-    Official HGNC gene name: HNF1 homeobox B
+    Alias gene symbol: D22S671
+    HGNC record ID: HGNC:4055
+    Primary gene symbol: XRCC6
+    Official HGNC gene name: X-ray repair cross complementing 6
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -695,16 +716,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "HPC11",
-    "primary_gene_symbol": "HNF1B",
-    "name": "HNF1 homeobox B",
+    "hgnc_id:"HGNC:4055"
+    "alias_symbol": "D22S671",
+    "primary_gene_symbol": "XRCC6",
+    "name": "X-ray repair cross complementing 6",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -712,10 +733,10 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "HPC11",
-"primary_gene_symbol": "HNF1B",
-"name": "HNF1 homeobox B",
+"hgnc_id": "HGNC:4055",
+"alias_symbol": "D22S671",
+"primary_gene_symbol": "XRCC6",
+"name": "X-ray repair cross complementing 6",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -724,32 +745,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HGNC:56665</t>
+          <t>HGNC:975</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ENSG00000231412</t>
+          <t>ENSG00000116752</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GENE ID:128193286</t>
+          <t>GENE ID:10286</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LINC03078</t>
+          <t>BCAS2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AC005392.2</t>
+          <t>SPF27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>long intergenic non-protein coding RNA 3078</t>
+          <t>BCAS2 pre-mRNA processing factor</t>
         </is>
       </c>
       <c r="G5" t="b">
@@ -759,14 +780,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: AC005392.2
-    HGNC record ID: HGNC:56665
-    Primary gene symbol: LINC03078
-    Official HGNC gene name: long intergenic non-protein coding RNA 3078
+    Alias gene symbol: SPF27
+    HGNC record ID: HGNC:975
+    Primary gene symbol: BCAS2
+    Official HGNC gene name: BCAS2 pre-mRNA processing factor
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -777,16 +805,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "AC005392.2",
-    "primary_gene_symbol": "LINC03078",
-    "name": "long intergenic non-protein coding RNA 3078",
+    "hgnc_id:"HGNC:975"
+    "alias_symbol": "SPF27",
+    "primary_gene_symbol": "BCAS2",
+    "name": "BCAS2 pre-mRNA processing factor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -794,10 +822,10 @@
       <c r="I5" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "AC005392.2",
-"primary_gene_symbol": "LINC03078",
-"name": "long intergenic non-protein coding RNA 3078",
+"hgnc_id": "HGNC:975",
+"alias_symbol": "SPF27",
+"primary_gene_symbol": "BCAS2",
+"name": "BCAS2 pre-mRNA processing factor",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -806,32 +834,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HGNC:15861</t>
+          <t>HGNC:6138</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ENSG00000101452</t>
+          <t>ENSG00000005961</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GENE ID:60625</t>
+          <t>GENE ID:3674</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DHX35</t>
+          <t>ITGA2B</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FLJ22759</t>
+          <t>GT1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DEAH-box helicase 35</t>
+          <t>integrin subunit alpha 2b</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -841,14 +869,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: FLJ22759
-    HGNC record ID: HGNC:15861
-    Primary gene symbol: DHX35
-    Official HGNC gene name: DEAH-box helicase 35
+    Alias gene symbol: GT1
+    HGNC record ID: HGNC:6138
+    Primary gene symbol: ITGA2B
+    Official HGNC gene name: integrin subunit alpha 2b
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -859,16 +894,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "FLJ22759",
-    "primary_gene_symbol": "DHX35",
-    "name": "DEAH-box helicase 35",
+    "hgnc_id:"HGNC:6138"
+    "alias_symbol": "GT1",
+    "primary_gene_symbol": "ITGA2B",
+    "name": "integrin subunit alpha 2b",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -876,10 +911,10 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "FLJ22759",
-"primary_gene_symbol": "DHX35",
-"name": "DEAH-box helicase 35",
+"hgnc_id": "HGNC:6138",
+"alias_symbol": "GT1",
+"primary_gene_symbol": "ITGA2B",
+"name": "integrin subunit alpha 2b",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -888,32 +923,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HGNC:28324</t>
+          <t>HGNC:23365</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ENSG00000167664</t>
+          <t>ENSG00000231293</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GENE ID:126259</t>
+          <t>set()</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TMIGD2</t>
+          <t>RPL36AP6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MGC23244</t>
+          <t>BA380I20.1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>transmembrane and immunoglobulin domain containing 2</t>
+          <t>ribosomal protein L36a pseudogene 6</t>
         </is>
       </c>
       <c r="G7" t="b">
@@ -923,14 +958,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: MGC23244
-    HGNC record ID: HGNC:28324
-    Primary gene symbol: TMIGD2
-    Official HGNC gene name: transmembrane and immunoglobulin domain containing 2
+    Alias gene symbol: BA380I20.1
+    HGNC record ID: HGNC:23365
+    Primary gene symbol: RPL36AP6
+    Official HGNC gene name: ribosomal protein L36a pseudogene 6
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -941,16 +983,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "MGC23244",
-    "primary_gene_symbol": "TMIGD2",
-    "name": "transmembrane and immunoglobulin domain containing 2",
+    "hgnc_id:"HGNC:23365"
+    "alias_symbol": "BA380I20.1",
+    "primary_gene_symbol": "RPL36AP6",
+    "name": "ribosomal protein L36a pseudogene 6",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -958,10 +1000,10 @@
       <c r="I7" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "MGC23244",
-"primary_gene_symbol": "TMIGD2",
-"name": "transmembrane and immunoglobulin domain containing 2",
+"hgnc_id": "HGNC:23365",
+"alias_symbol": "BA380I20.1",
+"primary_gene_symbol": "RPL36AP6",
+"name": "ribosomal protein L36a pseudogene 6",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -970,49 +1012,56 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HGNC:17284</t>
+          <t>HGNC:18656</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ENSG00000128513</t>
+          <t>ENSG00000124784</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GENE ID:25913</t>
+          <t>GENE ID:83732</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>POT1</t>
+          <t>RIOK1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>hPot1</t>
+          <t>AD034</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>protection of telomeres 1</t>
+          <t>RIO kinase 1</t>
         </is>
       </c>
       <c r="G8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: hPot1
-    HGNC record ID: HGNC:17284
-    Primary gene symbol: POT1
-    Official HGNC gene name: protection of telomeres 1
+    Alias gene symbol: AD034
+    HGNC record ID: HGNC:18656
+    Primary gene symbol: RIOK1
+    Official HGNC gene name: RIO kinase 1
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1023,16 +1072,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "hPot1",
-    "primary_gene_symbol": "POT1",
-    "name": "protection of telomeres 1",
+    "hgnc_id:"HGNC:18656"
+    "alias_symbol": "AD034",
+    "primary_gene_symbol": "RIOK1",
+    "name": "RIO kinase 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1040,11 +1089,11 @@
       <c r="I8" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "hPot1",
-"primary_gene_symbol": "POT1",
-"name": "protection of telomeres 1",
-"alternate_abbreviation": "TRUE"
+"hgnc_id": "HGNC:18656",
+"alias_symbol": "AD034",
+"primary_gene_symbol": "RIOK1",
+"name": "RIO kinase 1",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -1052,32 +1101,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HGNC:21238</t>
+          <t>HGNC:10924</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ENSG00000172738</t>
+          <t>ENSG00000141526</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GENE ID:221468</t>
+          <t>GENE ID:9123</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>TMEM217</t>
+          <t>SLC16A3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DJ355M6.2</t>
+          <t>MCT3</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>transmembrane protein 217</t>
+          <t>solute carrier family 16 member 3</t>
         </is>
       </c>
       <c r="G9" t="b">
@@ -1087,14 +1136,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: DJ355M6.2
-    HGNC record ID: HGNC:21238
-    Primary gene symbol: TMEM217
-    Official HGNC gene name: transmembrane protein 217
+    Alias gene symbol: MCT3
+    HGNC record ID: HGNC:10924
+    Primary gene symbol: SLC16A3
+    Official HGNC gene name: solute carrier family 16 member 3
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1105,16 +1161,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "DJ355M6.2",
-    "primary_gene_symbol": "TMEM217",
-    "name": "transmembrane protein 217",
+    "hgnc_id:"HGNC:10924"
+    "alias_symbol": "MCT3",
+    "primary_gene_symbol": "SLC16A3",
+    "name": "solute carrier family 16 member 3",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1122,10 +1178,10 @@
       <c r="I9" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "DJ355M6.2",
-"primary_gene_symbol": "TMEM217",
-"name": "transmembrane protein 217",
+"hgnc_id": "HGNC:10924",
+"alias_symbol": "MCT3",
+"primary_gene_symbol": "SLC16A3",
+"name": "solute carrier family 16 member 3",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1134,49 +1190,56 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HGNC:24845</t>
+          <t>HGNC:7406</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ENSG00000135631</t>
+          <t>ENSG00000125148</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GENE ID:26056</t>
+          <t>GENE ID:4502</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>RAB11FIP5</t>
+          <t>MT2A</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>pp75</t>
+          <t>MT-II</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>RAB11 family interacting protein 5</t>
+          <t>metallothionein 2A</t>
         </is>
       </c>
       <c r="G10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: pp75
-    HGNC record ID: HGNC:24845
-    Primary gene symbol: RAB11FIP5
-    Official HGNC gene name: RAB11 family interacting protein 5
+    Alias gene symbol: MT-II
+    HGNC record ID: HGNC:7406
+    Primary gene symbol: MT2A
+    Official HGNC gene name: metallothionein 2A
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1187,16 +1250,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "pp75",
-    "primary_gene_symbol": "RAB11FIP5",
-    "name": "RAB11 family interacting protein 5",
+    "hgnc_id:"HGNC:7406"
+    "alias_symbol": "MT-II",
+    "primary_gene_symbol": "MT2A",
+    "name": "metallothionein 2A",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1204,11 +1267,11 @@
       <c r="I10" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "pp75",
-"primary_gene_symbol": "RAB11FIP5",
-"name": "RAB11 family interacting protein 5",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:7406",
+"alias_symbol": "MT-II",
+"primary_gene_symbol": "MT2A",
+"name": "metallothionein 2A",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -1216,32 +1279,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HGNC:21916</t>
+          <t>HGNC:4790</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ENSG00000106125</t>
+          <t>ENSG00000276966</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GENE ID:84182</t>
+          <t>GENE ID:8367</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MINDY4</t>
+          <t>H4C5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FLJ22374</t>
+          <t>TEBIVANED3</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>MINDY lysine 48 deubiquitinase 4</t>
+          <t>H4 clustered histone 5</t>
         </is>
       </c>
       <c r="G11" t="b">
@@ -1251,14 +1314,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: FLJ22374
-    HGNC record ID: HGNC:21916
-    Primary gene symbol: MINDY4
-    Official HGNC gene name: MINDY lysine 48 deubiquitinase 4
+    Alias gene symbol: TEBIVANED3
+    HGNC record ID: HGNC:4790
+    Primary gene symbol: H4C5
+    Official HGNC gene name: H4 clustered histone 5
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1269,16 +1339,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "FLJ22374",
-    "primary_gene_symbol": "MINDY4",
-    "name": "MINDY lysine 48 deubiquitinase 4",
+    "hgnc_id:"HGNC:4790"
+    "alias_symbol": "TEBIVANED3",
+    "primary_gene_symbol": "H4C5",
+    "name": "H4 clustered histone 5",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1286,10 +1356,10 @@
       <c r="I11" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "FLJ22374",
-"primary_gene_symbol": "MINDY4",
-"name": "MINDY lysine 48 deubiquitinase 4",
+"hgnc_id": "HGNC:4790",
+"alias_symbol": "TEBIVANED3",
+"primary_gene_symbol": "H4C5",
+"name": "H4 clustered histone 5",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1298,49 +1368,56 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HGNC:7973</t>
+          <t>HGNC:31577</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ENSG00000112333</t>
+          <t>ENSG00000283762</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GENE ID:7101</t>
+          <t>GENE ID:406982</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NR2E1</t>
+          <t>MIR20A</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>XTLL</t>
+          <t>miR-20</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>nuclear receptor subfamily 2 group E member 1</t>
+          <t>microRNA 20a</t>
         </is>
       </c>
       <c r="G12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: XTLL
-    HGNC record ID: HGNC:7973
-    Primary gene symbol: NR2E1
-    Official HGNC gene name: nuclear receptor subfamily 2 group E member 1
+    Alias gene symbol: miR-20
+    HGNC record ID: HGNC:31577
+    Primary gene symbol: MIR20A
+    Official HGNC gene name: microRNA 20a
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1351,16 +1428,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "XTLL",
-    "primary_gene_symbol": "NR2E1",
-    "name": "nuclear receptor subfamily 2 group E member 1",
+    "hgnc_id:"HGNC:31577"
+    "alias_symbol": "miR-20",
+    "primary_gene_symbol": "MIR20A",
+    "name": "microRNA 20a",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1368,11 +1445,11 @@
       <c r="I12" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "XTLL",
-"primary_gene_symbol": "NR2E1",
-"name": "nuclear receptor subfamily 2 group E member 1",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:31577",
+"alias_symbol": "miR-20",
+"primary_gene_symbol": "MIR20A",
+"name": "microRNA 20a",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -1380,32 +1457,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HGNC:1366</t>
+          <t>HGNC:4516</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ENSG00000160323, ENSG00000281244</t>
+          <t>ENSG00000173698</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GENE ID:11093</t>
+          <t>GENE ID:10149</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ADAMTS13</t>
+          <t>ADGRG2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TTP</t>
+          <t>HE6</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ADAM metallopeptidase with thrombospondin type 1 motif 13</t>
+          <t>adhesion G protein-coupled receptor G2</t>
         </is>
       </c>
       <c r="G13" t="b">
@@ -1415,14 +1492,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: TTP
-    HGNC record ID: HGNC:1366
-    Primary gene symbol: ADAMTS13
-    Official HGNC gene name: ADAM metallopeptidase with thrombospondin type 1 motif 13
+    Alias gene symbol: HE6
+    HGNC record ID: HGNC:4516
+    Primary gene symbol: ADGRG2
+    Official HGNC gene name: adhesion G protein-coupled receptor G2
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1433,16 +1517,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "TTP",
-    "primary_gene_symbol": "ADAMTS13",
-    "name": "ADAM metallopeptidase with thrombospondin type 1 motif 13",
+    "hgnc_id:"HGNC:4516"
+    "alias_symbol": "HE6",
+    "primary_gene_symbol": "ADGRG2",
+    "name": "adhesion G protein-coupled receptor G2",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1450,10 +1534,10 @@
       <c r="I13" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "TTP",
-"primary_gene_symbol": "ADAMTS13",
-"name": "ADAM metallopeptidase with thrombospondin type 1 motif 13",
+"hgnc_id": "HGNC:4516",
+"alias_symbol": "HE6",
+"primary_gene_symbol": "ADGRG2",
+"name": "adhesion G protein-coupled receptor G2",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1462,49 +1546,56 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HGNC:5284</t>
+          <t>HGNC:32605</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ENSG00000205649</t>
+          <t>ENSG00000280498, ENSG00000274582</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GENE ID:3347</t>
+          <t>GENE ID:692073</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>HTN3</t>
+          <t>SNORA16A</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>HTN5</t>
+          <t>ACA16</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>histatin 3</t>
+          <t>small nucleolar RNA, H/ACA box 16A</t>
         </is>
       </c>
       <c r="G14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: HTN5
-    HGNC record ID: HGNC:5284
-    Primary gene symbol: HTN3
-    Official HGNC gene name: histatin 3
+    Alias gene symbol: ACA16
+    HGNC record ID: HGNC:32605
+    Primary gene symbol: SNORA16A
+    Official HGNC gene name: small nucleolar RNA, H/ACA box 16A
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1515,16 +1606,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "HTN5",
-    "primary_gene_symbol": "HTN3",
-    "name": "histatin 3",
+    "hgnc_id:"HGNC:32605"
+    "alias_symbol": "ACA16",
+    "primary_gene_symbol": "SNORA16A",
+    "name": "small nucleolar RNA, H/ACA box 16A",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1532,11 +1623,11 @@
       <c r="I14" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "HTN5",
-"primary_gene_symbol": "HTN3",
-"name": "histatin 3",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:32605",
+"alias_symbol": "ACA16",
+"primary_gene_symbol": "SNORA16A",
+"name": "small nucleolar RNA, H/ACA box 16A",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -1544,32 +1635,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HGNC:1555</t>
+          <t>HGNC:1514</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ENSG00000094916</t>
+          <t>ENSG00000036828</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GENE ID:23468</t>
+          <t>GENE ID:846</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CBX5</t>
+          <t>CASR</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HEL25</t>
+          <t>HHC</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>chromobox 5</t>
+          <t>calcium sensing receptor</t>
         </is>
       </c>
       <c r="G15" t="b">
@@ -1579,14 +1670,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: HEL25
-    HGNC record ID: HGNC:1555
-    Primary gene symbol: CBX5
-    Official HGNC gene name: chromobox 5
+    Alias gene symbol: HHC
+    HGNC record ID: HGNC:1514
+    Primary gene symbol: CASR
+    Official HGNC gene name: calcium sensing receptor
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1597,16 +1695,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "HEL25",
-    "primary_gene_symbol": "CBX5",
-    "name": "chromobox 5",
+    "hgnc_id:"HGNC:1514"
+    "alias_symbol": "HHC",
+    "primary_gene_symbol": "CASR",
+    "name": "calcium sensing receptor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1614,10 +1712,10 @@
       <c r="I15" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "HEL25",
-"primary_gene_symbol": "CBX5",
-"name": "chromobox 5",
+"hgnc_id": "HGNC:1514",
+"alias_symbol": "HHC",
+"primary_gene_symbol": "CASR",
+"name": "calcium sensing receptor",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1626,32 +1724,32 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HGNC:2372</t>
+          <t>HGNC:13994</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ENSG00000112282</t>
+          <t>ENSG00000164256</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GENE ID:9439</t>
+          <t>GENE ID:56979</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MED23</t>
+          <t>PRDM9</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>-SURæ2.00</t>
+          <t>Meisetz</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>mediator complex subunit 23</t>
+          <t>PR/SET domain 9</t>
         </is>
       </c>
       <c r="G16" t="b">
@@ -1661,14 +1759,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: -SURæ2.00
-    HGNC record ID: HGNC:2372
-    Primary gene symbol: MED23
-    Official HGNC gene name: mediator complex subunit 23
+    Alias gene symbol: Meisetz
+    HGNC record ID: HGNC:13994
+    Primary gene symbol: PRDM9
+    Official HGNC gene name: PR/SET domain 9
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1679,16 +1784,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "-SURæ2.00",
-    "primary_gene_symbol": "MED23",
-    "name": "mediator complex subunit 23",
+    "hgnc_id:"HGNC:13994"
+    "alias_symbol": "Meisetz",
+    "primary_gene_symbol": "PRDM9",
+    "name": "PR/SET domain 9",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1696,10 +1801,10 @@
       <c r="I16" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "-SURæ2.00",
-"primary_gene_symbol": "MED23",
-"name": "mediator complex subunit 23",
+"hgnc_id": "HGNC:13994",
+"alias_symbol": "Meisetz",
+"primary_gene_symbol": "PRDM9",
+"name": "PR/SET domain 9",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1708,32 +1813,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HGNC:5047</t>
+          <t>HGNC:41666</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ENSG00000125944</t>
+          <t>ENSG00000266517</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GENE ID:10236</t>
+          <t>GENE ID:100616474</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>HNRNPR</t>
+          <t>MIR4715</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NEDDFSB</t>
+          <t>HSA-MIR-4715</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>heterogeneous nuclear ribonucleoprotein R</t>
+          <t>microRNA 4715</t>
         </is>
       </c>
       <c r="G17" t="b">
@@ -1743,14 +1848,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: NEDDFSB
-    HGNC record ID: HGNC:5047
-    Primary gene symbol: HNRNPR
-    Official HGNC gene name: heterogeneous nuclear ribonucleoprotein R
+    Alias gene symbol: HSA-MIR-4715
+    HGNC record ID: HGNC:41666
+    Primary gene symbol: MIR4715
+    Official HGNC gene name: microRNA 4715
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1761,16 +1873,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "NEDDFSB",
-    "primary_gene_symbol": "HNRNPR",
-    "name": "heterogeneous nuclear ribonucleoprotein R",
+    "hgnc_id:"HGNC:41666"
+    "alias_symbol": "HSA-MIR-4715",
+    "primary_gene_symbol": "MIR4715",
+    "name": "microRNA 4715",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1778,10 +1890,10 @@
       <c r="I17" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "NEDDFSB",
-"primary_gene_symbol": "HNRNPR",
-"name": "heterogeneous nuclear ribonucleoprotein R",
+"hgnc_id": "HGNC:41666",
+"alias_symbol": "HSA-MIR-4715",
+"primary_gene_symbol": "MIR4715",
+"name": "microRNA 4715",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1790,49 +1902,56 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HGNC:10009</t>
+          <t>HGNC:8680</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ENSG00000187010</t>
+          <t>ENSG00000171815, ENSG00000291669</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GENE ID:6007</t>
+          <t>GENE ID:29930</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>RHD</t>
+          <t>PCDHB1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RHPII</t>
+          <t>PCDH-BETA1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Rh blood group D antigen</t>
+          <t>protocadherin beta 1</t>
         </is>
       </c>
       <c r="G18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: RHPII
-    HGNC record ID: HGNC:10009
-    Primary gene symbol: RHD
-    Official HGNC gene name: Rh blood group D antigen
+    Alias gene symbol: PCDH-BETA1
+    HGNC record ID: HGNC:8680
+    Primary gene symbol: PCDHB1
+    Official HGNC gene name: protocadherin beta 1
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1843,16 +1962,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "RHPII",
-    "primary_gene_symbol": "RHD",
-    "name": "Rh blood group D antigen",
+    "hgnc_id:"HGNC:8680"
+    "alias_symbol": "PCDH-BETA1",
+    "primary_gene_symbol": "PCDHB1",
+    "name": "protocadherin beta 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1860,11 +1979,11 @@
       <c r="I18" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "RHPII",
-"primary_gene_symbol": "RHD",
-"name": "Rh blood group D antigen",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:8680",
+"alias_symbol": "PCDH-BETA1",
+"primary_gene_symbol": "PCDHB1",
+"name": "protocadherin beta 1",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -1872,32 +1991,32 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HGNC:4250</t>
+          <t>HGNC:30422</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ENSG00000100031</t>
+          <t>ENSG00000138771</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GENE ID:2678</t>
+          <t>GENE ID:57619</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GGT1</t>
+          <t>SHROOM3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CD224</t>
+          <t>APXL3</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>gamma-glutamyltransferase 1</t>
+          <t>shroom family member 3</t>
         </is>
       </c>
       <c r="G19" t="b">
@@ -1907,14 +2026,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: CD224
-    HGNC record ID: HGNC:4250
-    Primary gene symbol: GGT1
-    Official HGNC gene name: gamma-glutamyltransferase 1
+    Alias gene symbol: APXL3
+    HGNC record ID: HGNC:30422
+    Primary gene symbol: SHROOM3
+    Official HGNC gene name: shroom family member 3
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1925,16 +2051,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "CD224",
-    "primary_gene_symbol": "GGT1",
-    "name": "gamma-glutamyltransferase 1",
+    "hgnc_id:"HGNC:30422"
+    "alias_symbol": "APXL3",
+    "primary_gene_symbol": "SHROOM3",
+    "name": "shroom family member 3",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1942,10 +2068,10 @@
       <c r="I19" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "CD224",
-"primary_gene_symbol": "GGT1",
-"name": "gamma-glutamyltransferase 1",
+"hgnc_id": "HGNC:30422",
+"alias_symbol": "APXL3",
+"primary_gene_symbol": "SHROOM3",
+"name": "shroom family member 3",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1954,32 +2080,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HGNC:7127</t>
+          <t>HGNC:17284</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ENSG00000076242</t>
+          <t>ENSG00000128513</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GENE ID:4292</t>
+          <t>GENE ID:25913</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MLH1</t>
+          <t>POT1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MMRCS1</t>
+          <t>hPot1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>mutL homolog 1</t>
+          <t>protection of telomeres 1</t>
         </is>
       </c>
       <c r="G20" t="b">
@@ -1989,14 +2115,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: MMRCS1
-    HGNC record ID: HGNC:7127
-    Primary gene symbol: MLH1
-    Official HGNC gene name: mutL homolog 1
+    Alias gene symbol: hPot1
+    HGNC record ID: HGNC:17284
+    Primary gene symbol: POT1
+    Official HGNC gene name: protection of telomeres 1
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2007,16 +2140,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "MMRCS1",
-    "primary_gene_symbol": "MLH1",
-    "name": "mutL homolog 1",
+    "hgnc_id:"HGNC:17284"
+    "alias_symbol": "hPot1",
+    "primary_gene_symbol": "POT1",
+    "name": "protection of telomeres 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2024,11 +2157,11 @@
       <c r="I20" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "MMRCS1",
-"primary_gene_symbol": "MLH1",
-"name": "mutL homolog 1",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:17284",
+"alias_symbol": "hPot1",
+"primary_gene_symbol": "POT1",
+"name": "protection of telomeres 1",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -2036,32 +2169,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HGNC:19336</t>
+          <t>HGNC:13243</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ENSG00000146414</t>
+          <t>ENSG00000105983</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GENE ID:257218</t>
+          <t>GENE ID:64327</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>SHPRH</t>
+          <t>LMBR1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BA545I5.2</t>
+          <t>PPD2</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SNF2 histone linker PHD RING helicase</t>
+          <t>limb development membrane protein 1</t>
         </is>
       </c>
       <c r="G21" t="b">
@@ -2071,14 +2204,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: BA545I5.2
-    HGNC record ID: HGNC:19336
-    Primary gene symbol: SHPRH
-    Official HGNC gene name: SNF2 histone linker PHD RING helicase
+    Alias gene symbol: PPD2
+    HGNC record ID: HGNC:13243
+    Primary gene symbol: LMBR1
+    Official HGNC gene name: limb development membrane protein 1
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2089,16 +2229,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "BA545I5.2",
-    "primary_gene_symbol": "SHPRH",
-    "name": "SNF2 histone linker PHD RING helicase",
+    "hgnc_id:"HGNC:13243"
+    "alias_symbol": "PPD2",
+    "primary_gene_symbol": "LMBR1",
+    "name": "limb development membrane protein 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2106,10 +2246,10 @@
       <c r="I21" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "BA545I5.2",
-"primary_gene_symbol": "SHPRH",
-"name": "SNF2 histone linker PHD RING helicase",
+"hgnc_id": "HGNC:13243",
+"alias_symbol": "PPD2",
+"primary_gene_symbol": "LMBR1",
+"name": "limb development membrane protein 1",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -2118,32 +2258,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HGNC:10963</t>
+          <t>HGNC:330</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ENSG00000175003</t>
+          <t>ENSG00000159723</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GENE ID:6580</t>
+          <t>GENE ID:181</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SLC22A1</t>
+          <t>AGRP</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>HOCT1</t>
+          <t>ASIP2</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>solute carrier family 22 member 1</t>
+          <t>agouti related neuropeptide</t>
         </is>
       </c>
       <c r="G22" t="b">
@@ -2153,14 +2293,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: HOCT1
-    HGNC record ID: HGNC:10963
-    Primary gene symbol: SLC22A1
-    Official HGNC gene name: solute carrier family 22 member 1
+    Alias gene symbol: ASIP2
+    HGNC record ID: HGNC:330
+    Primary gene symbol: AGRP
+    Official HGNC gene name: agouti related neuropeptide
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2171,16 +2318,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "HOCT1",
-    "primary_gene_symbol": "SLC22A1",
-    "name": "solute carrier family 22 member 1",
+    "hgnc_id:"HGNC:330"
+    "alias_symbol": "ASIP2",
+    "primary_gene_symbol": "AGRP",
+    "name": "agouti related neuropeptide",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2188,10 +2335,10 @@
       <c r="I22" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "HOCT1",
-"primary_gene_symbol": "SLC22A1",
-"name": "solute carrier family 22 member 1",
+"hgnc_id": "HGNC:330",
+"alias_symbol": "ASIP2",
+"primary_gene_symbol": "AGRP",
+"name": "agouti related neuropeptide",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -2200,32 +2347,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HGNC:25945</t>
+          <t>HGNC:26435</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ENSG00000185305</t>
+          <t>ENSG00000276914, ENSG00000133393</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GENE ID:54622</t>
+          <t>GENE ID:123811</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ARLæ15.00</t>
+          <t>CEP20</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FLJ20051</t>
+          <t>FOR20</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>ARF like GTPase 15</t>
+          <t>centrosomal protein 20</t>
         </is>
       </c>
       <c r="G23" t="b">
@@ -2235,14 +2382,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: FLJ20051
-    HGNC record ID: HGNC:25945
-    Primary gene symbol: ARLæ15.00
-    Official HGNC gene name: ARF like GTPase 15
+    Alias gene symbol: FOR20
+    HGNC record ID: HGNC:26435
+    Primary gene symbol: CEP20
+    Official HGNC gene name: centrosomal protein 20
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2253,16 +2407,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "FLJ20051",
-    "primary_gene_symbol": "ARLæ15.00",
-    "name": "ARF like GTPase 15",
+    "hgnc_id:"HGNC:26435"
+    "alias_symbol": "FOR20",
+    "primary_gene_symbol": "CEP20",
+    "name": "centrosomal protein 20",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2270,10 +2424,10 @@
       <c r="I23" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "FLJ20051",
-"primary_gene_symbol": "ARLæ15.00",
-"name": "ARF like GTPase 15",
+"hgnc_id": "HGNC:26435",
+"alias_symbol": "FOR20",
+"primary_gene_symbol": "CEP20",
+"name": "centrosomal protein 20",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -2282,49 +2436,56 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HGNC:17005</t>
+          <t>HGNC:32625</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ENSG00000136110</t>
+          <t>ENSG00000208839</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GENE ID:11061</t>
+          <t>GENE ID:677816</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CNMD</t>
+          <t>SNORA35</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CHM-I</t>
+          <t>HBI-36</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>chondromodulin</t>
+          <t>small nucleolar RNA, H/ACA box 35</t>
         </is>
       </c>
       <c r="G24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: CHM-I
-    HGNC record ID: HGNC:17005
-    Primary gene symbol: CNMD
-    Official HGNC gene name: chondromodulin
+    Alias gene symbol: HBI-36
+    HGNC record ID: HGNC:32625
+    Primary gene symbol: SNORA35
+    Official HGNC gene name: small nucleolar RNA, H/ACA box 35
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2335,16 +2496,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "CHM-I",
-    "primary_gene_symbol": "CNMD",
-    "name": "chondromodulin",
+    "hgnc_id:"HGNC:32625"
+    "alias_symbol": "HBI-36",
+    "primary_gene_symbol": "SNORA35",
+    "name": "small nucleolar RNA, H/ACA box 35",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2352,11 +2513,11 @@
       <c r="I24" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "CHM-I",
-"primary_gene_symbol": "CNMD",
-"name": "chondromodulin",
-"alternate_abbreviation": "TRUE"
+"hgnc_id": "HGNC:32625",
+"alias_symbol": "HBI-36",
+"primary_gene_symbol": "SNORA35",
+"name": "small nucleolar RNA, H/ACA box 35",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -2364,49 +2525,56 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HGNC:36791</t>
+          <t>HGNC:13525</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>set()</t>
+          <t>ENSG00000242950</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GENE ID:100271646</t>
+          <t>GENE ID:30816</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RPL36AP43</t>
+          <t>ERVW-1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RPL36A_21_1460</t>
+          <t>HERV-7Q</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ribosomal protein L36a pseudogene 43</t>
+          <t>endogenous retrovirus group W member 1, envelope</t>
         </is>
       </c>
       <c r="G25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: RPL36A_21_1460
-    HGNC record ID: HGNC:36791
-    Primary gene symbol: RPL36AP43
-    Official HGNC gene name: ribosomal protein L36a pseudogene 43
+    Alias gene symbol: HERV-7Q
+    HGNC record ID: HGNC:13525
+    Primary gene symbol: ERVW-1
+    Official HGNC gene name: endogenous retrovirus group W member 1, envelope
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2417,16 +2585,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "RPL36A_21_1460",
-    "primary_gene_symbol": "RPL36AP43",
-    "name": "ribosomal protein L36a pseudogene 43",
+    "hgnc_id:"HGNC:13525"
+    "alias_symbol": "HERV-7Q",
+    "primary_gene_symbol": "ERVW-1",
+    "name": "endogenous retrovirus group W member 1, envelope",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2434,10 +2602,10 @@
       <c r="I25" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "RPL36A_21_1460",
-"primary_gene_symbol": "RPL36AP43",
-"name": "ribosomal protein L36a pseudogene 43",
+"hgnc_id": "HGNC:13525",
+"alias_symbol": "HERV-7Q",
+"primary_gene_symbol": "ERVW-1",
+"name": "endogenous retrovirus group W member 1, envelope",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -2446,49 +2614,56 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HGNC:3595</t>
+          <t>HGNC:18001</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ENSG00000083857</t>
+          <t>ENSG00000130204</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GENE ID:2195</t>
+          <t>GENE ID:10452</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>FAT1</t>
+          <t>TOMM40</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FAT</t>
+          <t>PEREC1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>FAT atypical cadherin 1</t>
+          <t>translocase of outer mitochondrial membrane 40</t>
         </is>
       </c>
       <c r="G26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: FAT
-    HGNC record ID: HGNC:3595
-    Primary gene symbol: FAT1
-    Official HGNC gene name: FAT atypical cadherin 1
+    Alias gene symbol: PEREC1
+    HGNC record ID: HGNC:18001
+    Primary gene symbol: TOMM40
+    Official HGNC gene name: translocase of outer mitochondrial membrane 40
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2499,16 +2674,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "FAT",
-    "primary_gene_symbol": "FAT1",
-    "name": "FAT atypical cadherin 1",
+    "hgnc_id:"HGNC:18001"
+    "alias_symbol": "PEREC1",
+    "primary_gene_symbol": "TOMM40",
+    "name": "translocase of outer mitochondrial membrane 40",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2516,10 +2691,10 @@
       <c r="I26" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "FAT",
-"primary_gene_symbol": "FAT1",
-"name": "FAT atypical cadherin 1",
+"hgnc_id": "HGNC:18001",
+"alias_symbol": "PEREC1",
+"primary_gene_symbol": "TOMM40",
+"name": "translocase of outer mitochondrial membrane 40",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -2528,49 +2703,56 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>HGNC:29145</t>
+          <t>HGNC:3595</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ENSG00000132680</t>
+          <t>ENSG00000083857</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GENE ID:22889</t>
+          <t>GENE ID:2195</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>KHDC4</t>
+          <t>FAT1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SNORA80EHG</t>
+          <t>FAT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>KH domain containing 4, pre-mRNA splicing factor</t>
+          <t>FAT atypical cadherin 1</t>
         </is>
       </c>
       <c r="G27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: SNORA80EHG
-    HGNC record ID: HGNC:29145
-    Primary gene symbol: KHDC4
-    Official HGNC gene name: KH domain containing 4, pre-mRNA splicing factor
+    Alias gene symbol: FAT
+    HGNC record ID: HGNC:3595
+    Primary gene symbol: FAT1
+    Official HGNC gene name: FAT atypical cadherin 1
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2581,16 +2763,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "SNORA80EHG",
-    "primary_gene_symbol": "KHDC4",
-    "name": "KH domain containing 4, pre-mRNA splicing factor",
+    "hgnc_id:"HGNC:3595"
+    "alias_symbol": "FAT",
+    "primary_gene_symbol": "FAT1",
+    "name": "FAT atypical cadherin 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2598,11 +2780,11 @@
       <c r="I27" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "SNORA80EHG",
-"primary_gene_symbol": "KHDC4",
-"name": "KH domain containing 4, pre-mRNA splicing factor",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:3595",
+"alias_symbol": "FAT",
+"primary_gene_symbol": "FAT1",
+"name": "FAT atypical cadherin 1",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -2610,49 +2792,56 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>HGNC:32522</t>
+          <t>HGNC:5969</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ENSG00000182487, ENSG00000290838</t>
+          <t>ENSG00000168811</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GENE ID:654816</t>
+          <t>GENE ID:3592</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NCF1B</t>
+          <t>IL12A</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SH3PXD1B</t>
+          <t>IL-12A</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>neutrophil cytosolic factor 1B (pseudogene)</t>
+          <t>interleukin 12A</t>
         </is>
       </c>
       <c r="G28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: SH3PXD1B
-    HGNC record ID: HGNC:32522
-    Primary gene symbol: NCF1B
-    Official HGNC gene name: neutrophil cytosolic factor 1B (pseudogene)
+    Alias gene symbol: IL-12A
+    HGNC record ID: HGNC:5969
+    Primary gene symbol: IL12A
+    Official HGNC gene name: interleukin 12A
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2663,16 +2852,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "SH3PXD1B",
-    "primary_gene_symbol": "NCF1B",
-    "name": "neutrophil cytosolic factor 1B (pseudogene)",
+    "hgnc_id:"HGNC:5969"
+    "alias_symbol": "IL-12A",
+    "primary_gene_symbol": "IL12A",
+    "name": "interleukin 12A",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2680,11 +2869,11 @@
       <c r="I28" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "SH3PXD1B",
-"primary_gene_symbol": "NCF1B",
-"name": "neutrophil cytosolic factor 1B (pseudogene)",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:5969",
+"alias_symbol": "IL-12A",
+"primary_gene_symbol": "IL12A",
+"name": "interleukin 12A",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -2692,32 +2881,32 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HGNC:4872</t>
+          <t>HGNC:38178</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ENSG00000230267</t>
+          <t>set()</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GENE ID:100289574</t>
+          <t>GENE ID:100423041</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>HERC2P4</t>
+          <t>MIR4296</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>D16F37S5</t>
+          <t>hsa-mir-4296</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>HERC2 pseudogene 4</t>
+          <t>microRNA 4296</t>
         </is>
       </c>
       <c r="G29" t="b">
@@ -2727,14 +2916,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: D16F37S5
-    HGNC record ID: HGNC:4872
-    Primary gene symbol: HERC2P4
-    Official HGNC gene name: HERC2 pseudogene 4
+    Alias gene symbol: hsa-mir-4296
+    HGNC record ID: HGNC:38178
+    Primary gene symbol: MIR4296
+    Official HGNC gene name: microRNA 4296
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2745,16 +2941,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "D16F37S5",
-    "primary_gene_symbol": "HERC2P4",
-    "name": "HERC2 pseudogene 4",
+    "hgnc_id:"HGNC:38178"
+    "alias_symbol": "hsa-mir-4296",
+    "primary_gene_symbol": "MIR4296",
+    "name": "microRNA 4296",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2762,10 +2958,10 @@
       <c r="I29" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "D16F37S5",
-"primary_gene_symbol": "HERC2P4",
-"name": "HERC2 pseudogene 4",
+"hgnc_id": "HGNC:38178",
+"alias_symbol": "hsa-mir-4296",
+"primary_gene_symbol": "MIR4296",
+"name": "microRNA 4296",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -2774,49 +2970,56 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>HGNC:8944</t>
+          <t>HGNC:7505</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ENSG00000197641</t>
+          <t>ENSG00000236675</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GENE ID:5275</t>
+          <t>GENE ID:4581</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SERPINB13</t>
+          <t>MTX1LP</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>HUR7</t>
+          <t>psMTX</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>serpin family B member 13</t>
+          <t>metaxin 1 like, pseudogene</t>
         </is>
       </c>
       <c r="G30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: HUR7
-    HGNC record ID: HGNC:8944
-    Primary gene symbol: SERPINB13
-    Official HGNC gene name: serpin family B member 13
+    Alias gene symbol: psMTX
+    HGNC record ID: HGNC:7505
+    Primary gene symbol: MTX1LP
+    Official HGNC gene name: metaxin 1 like, pseudogene
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2827,16 +3030,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "HUR7",
-    "primary_gene_symbol": "SERPINB13",
-    "name": "serpin family B member 13",
+    "hgnc_id:"HGNC:7505"
+    "alias_symbol": "psMTX",
+    "primary_gene_symbol": "MTX1LP",
+    "name": "metaxin 1 like, pseudogene",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2844,11 +3047,11 @@
       <c r="I30" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "HUR7",
-"primary_gene_symbol": "SERPINB13",
-"name": "serpin family B member 13",
-"alternate_abbreviation": "FALSE"
+"hgnc_id": "HGNC:7505",
+"alias_symbol": "psMTX",
+"primary_gene_symbol": "MTX1LP",
+"name": "metaxin 1 like, pseudogene",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -2856,32 +3059,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HGNC:9911</t>
+          <t>HGNC:25338</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ENSG00000216835</t>
+          <t>ENSG00000139200</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GENE ID:3186</t>
+          <t>GENE ID:196500</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>RBMXP1</t>
+          <t>PIANP</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>HNRNP-G</t>
+          <t>DKFZP547D2210</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>RBMX pseudogene 1</t>
+          <t>PILR alpha associated neural protein</t>
         </is>
       </c>
       <c r="G31" t="b">
@@ -2891,14 +3094,21 @@
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: HNRNP-G
-    HGNC record ID: HGNC:9911
-    Primary gene symbol: RBMXP1
-    Official HGNC gene name: RBMX pseudogene 1
+    Alias gene symbol: DKFZP547D2210
+    HGNC record ID: HGNC:25338
+    Primary gene symbol: PIANP
+    Official HGNC gene name: PILR alpha associated neural protein
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
-    HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
+    HGNC gene name, or to a phrase that is nearly identical in wording and meaning. 
+    Another way to classify the alias symbol as an Alternate Abbreviation is to compare it to the primary gene symbol. If the only differences 
+    are nonalphanumeric characters, then the alias symbol is an Alternate Abbreviation.
+    If the alias is a simpler form of the primary gene symbol, missing some components of the gene name, then it is an Alternate Abbreviation.
+    If the alias is a more complex form of the primary gene symbol, adding numbers that are not reflected in the gene name, it is not an Alternate Abbreviation.
+    There is a special case of alias symbols for microRNA genes. These aliases include the primary gene symbol with a dash between the alphabetic and the numeric
+    characters and a three letter prefix. These aliases with the "hsa" or "HSA" prefix look like Alternate Abbreviations but are not. While those without 
+    the "hsa" or "HSA" are Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -2909,16 +3119,16 @@
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Primary gene symbol: A4GNT
     Rules:
-    If the text does not support that the alias is an alternate abbreviation, return:
+    If the alias is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "pmid": "",
-    "alias_symbol": "HNRNP-G",
-    "primary_gene_symbol": "RBMXP1",
-    "name": "RBMX pseudogene 1",
+    "hgnc_id:"HGNC:25338"
+    "alias_symbol": "DKFZP547D2210",
+    "primary_gene_symbol": "PIANP",
+    "name": "PILR alpha associated neural protein",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2926,10 +3136,10 @@
       <c r="I31" t="inlineStr">
         <is>
           <t>{
-"pmid": "",
-"alias_symbol": "HNRNP-G",
-"primary_gene_symbol": "RBMXP1",
-"name": "RBMX pseudogene 1",
+"hgnc_id": "HGNC:25338",
+"alias_symbol": "DKFZP547D2210",
+"primary_gene_symbol": "PIANP",
+"name": "PILR alpha associated neural protein",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>

</xml_diff>